<commit_message>
Subscripts SoICETAF by industry cat
</commit_message>
<xml_diff>
--- a/InputData/indst/SoICETAF/Share of Indst Cap Expenditures That Are Financed.xlsx
+++ b/InputData/indst/SoICETAF/Share of Indst Cap Expenditures That Are Financed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\indst\SoICETAF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F57A19-47D2-443A-B6DD-A3D65075AF37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2E009A-2237-4067-84F8-589D1EDA0408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10060" yWindow="950" windowWidth="14400" windowHeight="8210" tabRatio="644" xr2:uid="{C8F9D547-902B-4E49-8BA2-E23B0A2DC1A9}"/>
+    <workbookView xWindow="7155" yWindow="855" windowWidth="18390" windowHeight="11010" tabRatio="644" xr2:uid="{C8F9D547-902B-4E49-8BA2-E23B0A2DC1A9}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Source:</t>
   </si>
@@ -44,9 +44,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>industry-wide</t>
-  </si>
-  <si>
     <t>SoICETAF Share of Industry Capital Expenditures That Are Financed</t>
   </si>
   <si>
@@ -63,6 +60,81 @@
   </si>
   <si>
     <t>share</t>
+  </si>
+  <si>
+    <t>agriculture and forestry 01T03</t>
+  </si>
+  <si>
+    <t>coal mining 05</t>
+  </si>
+  <si>
+    <t>oil and gas extraction 06</t>
+  </si>
+  <si>
+    <t>other mining and quarrying 07T08</t>
+  </si>
+  <si>
+    <t>food beverage and tobacco 10T12</t>
+  </si>
+  <si>
+    <t>textiles apparel and leather 13T15</t>
+  </si>
+  <si>
+    <t>wood products 16</t>
+  </si>
+  <si>
+    <t>pulp paper and printing 17T18</t>
+  </si>
+  <si>
+    <t>refined petroleum and coke 19</t>
+  </si>
+  <si>
+    <t>chemicals 20</t>
+  </si>
+  <si>
+    <t>rubber and plastic products 22</t>
+  </si>
+  <si>
+    <t>glass and glass products 231</t>
+  </si>
+  <si>
+    <t>construction 41T43</t>
+  </si>
+  <si>
+    <t>cement and other nonmetallic minerals 239</t>
+  </si>
+  <si>
+    <t>iron and steel 241</t>
+  </si>
+  <si>
+    <t>other metals 242</t>
+  </si>
+  <si>
+    <t>metal products except machinery and vehicles 25</t>
+  </si>
+  <si>
+    <t>computers and electronics 26</t>
+  </si>
+  <si>
+    <t>appliances and electrical equipment 27</t>
+  </si>
+  <si>
+    <t>other machinery 28</t>
+  </si>
+  <si>
+    <t>road vehicles 29</t>
+  </si>
+  <si>
+    <t>nonroad vehicles 30</t>
+  </si>
+  <si>
+    <t>other manufacturing 31T33</t>
+  </si>
+  <si>
+    <t>energy pipelines and gas processing 352T353</t>
+  </si>
+  <si>
+    <t>water and waste 36T39</t>
   </si>
 </sst>
 </file>
@@ -482,46 +554,46 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23F0629E-7DF7-4E6A-B1DA-78D3050B5FAD}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="87.1796875" customWidth="1"/>
+    <col min="2" max="2" width="87.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -534,27 +606,219 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.1796875" customWidth="1"/>
+    <col min="1" max="1" width="38.140625" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="5" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
       <c r="B2" s="7">
-        <v>0.5</v>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26">
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>